<commit_message>
July 3 dates, cat-friendly + trailer-checked hotels, atlas label fixes
</commit_message>
<xml_diff>
--- a/cost-tracker.xlsx
+++ b/cost-tracker.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="88">
   <si>
     <t xml:space="preserve">Salina, KS  -&gt;  Leesburg, FL  ·  Move Itinerary</t>
   </si>
   <si>
-    <t xml:space="preserve">Departing Friday, July 10, 2026 · 4 days / 3 nights · 2018 Tacoma TRD (towing 2,300 lb T-bucket) + 2024 Land Cruiser · baby aboard</t>
+    <t xml:space="preserve">Departing Friday, July 3, 2026 (July 4th weekend) · cats · 4 days / 3 nights · 2018 Tacoma TRD (towing 2,300 lb T-bucket) + 2024 Land Cruiser · baby aboard</t>
   </si>
   <si>
     <t xml:space="preserve">Route (easiest towing): I-135 &gt; I-35 &gt; I-40 &gt; I-22 &gt; I-65 &gt; US-231 &gt; I-10 &gt; I-75 (Exit 329 Wildwood) · ~1,555 mi · ~23.5 hrs · $0 tolls</t>
@@ -54,7 +54,7 @@
     <t xml:space="preserve">Key highways</t>
   </si>
   <si>
-    <t xml:space="preserve">Jul 10</t>
+    <t xml:space="preserve">Jul 3</t>
   </si>
   <si>
     <t xml:space="preserve">Salina, KS</t>
@@ -66,7 +66,7 @@
     <t xml:space="preserve">I-135 S &gt; I-35 S</t>
   </si>
   <si>
-    <t xml:space="preserve">Jul 11</t>
+    <t xml:space="preserve">Jul 4</t>
   </si>
   <si>
     <t xml:space="preserve">Memphis, TN (East/Wolfchase)</t>
@@ -75,7 +75,7 @@
     <t xml:space="preserve">I-40 E (via Little Rock)</t>
   </si>
   <si>
-    <t xml:space="preserve">Jul 12</t>
+    <t xml:space="preserve">Jul 5</t>
   </si>
   <si>
     <t xml:space="preserve">Memphis, TN</t>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">I-22 E &gt; I-65 S</t>
   </si>
   <si>
-    <t xml:space="preserve">Jul 13</t>
+    <t xml:space="preserve">Jul 6</t>
   </si>
   <si>
     <t xml:space="preserve">Montgomery, AL</t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">Hotel Options - Marriott / Hilton family · on Hotels.com (use points)</t>
   </si>
   <si>
-    <t xml:space="preserve">Click a hotel name to open Hotels.com (use points). Mark one 'x' per night in Choose. Default picks pre-filled. Rooms/night editable (yellow).</t>
+    <t xml:space="preserve">July 4th-weekend rates - book early. All cat-friendly (~$50-75 pet fee). Click a hotel name to open Hotels.com. Mark one 'x' per night in Choose. Default picks pre-filled. Rooms/night editable (yellow).</t>
   </si>
   <si>
     <t xml:space="preserve">Rooms per night:</t>
@@ -201,37 +201,37 @@
     <t xml:space="preserve">x</t>
   </si>
   <si>
-    <t xml:space="preserve">OKC · I-40 @ Meridian</t>
+    <t xml:space="preserve">OKC · I-40/I-44 Meridian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hilton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.7/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats OK; RV/bus/truck parking; all-suite+kitchen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OKC · Meridian Row</t>
   </si>
   <si>
     <t xml:space="preserve">Marriott</t>
   </si>
   <si>
-    <t xml:space="preserve">3.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bus/horse-trailer parking; outdoor pool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OKC · I-40/I-44 Meridian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hilton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.7/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All-suite+kitchen; FREE bkfst; indoor pool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OKC · Meridian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.1/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FREE hot bkfst; indoor pool; shuttle</t>
+    <t xml:space="preserve">4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats OK; flat lot; suite+kitchen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OKC · behind row</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats OK; lot fills early; suite+kitchen</t>
   </si>
   <si>
     <t xml:space="preserve">Memphis E · I-40 Exit 16</t>
@@ -240,49 +240,43 @@
     <t xml:space="preserve">4.0+</t>
   </si>
   <si>
-    <t xml:space="preserve">Indoor saltwater pool; big-box lot</t>
+    <t xml:space="preserve">Cats OK; big standalone lot; indoor pool</t>
   </si>
   <si>
     <t xml:space="preserve">4.0</t>
   </si>
   <si>
-    <t xml:space="preserve">Patrolled lot; FREE hot bkfst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memphis E · Germantown Pkwy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indoor pool; Starbucks lobby</t>
+    <t xml:space="preserve">Cats OK; large free lot; FREE bkfst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Memphis · Germantown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats OK; smaller lot (fills eve); suite+kitchen</t>
   </si>
   <si>
     <t xml:space="preserve">Montgomery · I-85 EastChase</t>
   </si>
   <si>
+    <t xml:space="preserve">Cats OK; flat lot often empty (best for trailer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Montgomery · I-85 Exit 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.9/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cats OK; free surface lot; pool</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.7</t>
   </si>
   <si>
-    <t xml:space="preserve">Best of trip; FREE bkfst; huge lot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montgomery · I-85 Exit 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.9/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closest to East Blvd/I-65; pool</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Montgomery · I-85 Exit 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.9/10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parking on 3 sides; outdoor pool</t>
+    <t xml:space="preserve">Cats OK; buses OK but lot on steep hill</t>
   </si>
   <si>
     <t xml:space="preserve">Selected /night sum:</t>
@@ -1073,7 +1067,7 @@
       </c>
       <c r="B15" s="12" t="n">
         <f aca="false">Hotels!H20</f>
-        <v>796</v>
+        <v>968</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1095,7 +1089,7 @@
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">B14+B15+B16</f>
-        <v>1441.14517006803</v>
+        <v>1613.14517006803</v>
       </c>
     </row>
   </sheetData>
@@ -1322,7 +1316,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
         <v>58</v>
       </c>
@@ -1333,8 +1327,8 @@
         <v>59</v>
       </c>
       <c r="D7" s="33" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Courtyard%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","Courtyard OKC Airport")</f>
-        <v>Courtyard OKC Airport</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Home2%20Suites%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","Home2 Suites OKC Airport")</f>
+        <v>Home2 Suites OKC Airport</v>
       </c>
       <c r="E7" s="32" t="s">
         <v>60</v>
@@ -1343,7 +1337,7 @@
         <v>61</v>
       </c>
       <c r="G7" s="34" t="n">
-        <v>128</v>
+        <v>152</v>
       </c>
       <c r="H7" s="32" t="s">
         <v>62</v>
@@ -1358,8 +1352,8 @@
         <v>63</v>
       </c>
       <c r="D8" s="36" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Home2%20Suites%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","Home2 Suites OKC Airport")</f>
-        <v>Home2 Suites OKC Airport</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=TownePlace%20Suites%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","TownePlace Suites OKC Airport")</f>
+        <v>TownePlace Suites OKC Airport</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>64</v>
@@ -1368,7 +1362,7 @@
         <v>65</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>132</v>
+        <v>150</v>
       </c>
       <c r="H8" s="6" t="s">
         <v>66</v>
@@ -1383,17 +1377,17 @@
         <v>67</v>
       </c>
       <c r="D9" s="36" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Fairfield%20Inn%20%26%20Suites%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","Fairfield Inn &amp; Suites OKC Airport")</f>
-        <v>Fairfield Inn &amp; Suites OKC Airport</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Residence%20Inn%20OKC%20Airport%2C%20Oklahoma%20City%2C%20OK","Residence Inn OKC Airport")</f>
+        <v>Residence Inn OKC Airport</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>68</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>122</v>
+        <v>168</v>
       </c>
       <c r="H9" s="6" t="s">
         <v>69</v>
@@ -1414,13 +1408,13 @@
         <v>Hilton Garden Inn Wolfchase</v>
       </c>
       <c r="E10" s="32" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F10" s="31" t="s">
         <v>71</v>
       </c>
       <c r="G10" s="34" t="n">
-        <v>130</v>
+        <v>176</v>
       </c>
       <c r="H10" s="32" t="s">
         <v>72</v>
@@ -1439,13 +1433,13 @@
         <v>Hampton Inn &amp; Suites Wolfchase</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>73</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>130</v>
+        <v>172</v>
       </c>
       <c r="H11" s="6" t="s">
         <v>74</v>
@@ -1460,17 +1454,17 @@
         <v>75</v>
       </c>
       <c r="D12" s="36" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Courtyard%20Memphis%20Germantown%2C%20Memphis%2C%20TN","Courtyard Memphis Germantown")</f>
-        <v>Courtyard Memphis Germantown</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Residence%20Inn%20Memphis%20Germantown%2C%20Memphis%2C%20TN","Residence Inn Memphis Germantown")</f>
+        <v>Residence Inn Memphis Germantown</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F12" s="5" t="s">
         <v>76</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>125</v>
+        <v>180</v>
       </c>
       <c r="H12" s="6" t="s">
         <v>77</v>
@@ -1487,20 +1481,20 @@
         <v>78</v>
       </c>
       <c r="D13" s="33" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Hampton%20Inn%20%26%20Suites%20EastChase%2C%20Montgomery%2C%20AL","Hampton Inn &amp; Suites EastChase")</f>
-        <v>Hampton Inn &amp; Suites EastChase</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=TownePlace%20Suites%20Montgomery%20EastChase%2C%20Montgomery%2C%20AL","TownePlace Suites Montgomery EastChase")</f>
+        <v>TownePlace Suites Montgomery EastChase</v>
       </c>
       <c r="E13" s="32" t="s">
         <v>64</v>
       </c>
       <c r="F13" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>156</v>
+      </c>
+      <c r="H13" s="32" t="s">
         <v>79</v>
-      </c>
-      <c r="G13" s="34" t="n">
-        <v>140</v>
-      </c>
-      <c r="H13" s="32" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1509,23 +1503,23 @@
         <v>3</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D14" s="36" t="str">
         <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Hilton%20Garden%20Inn%20Montgomery%20East%2C%20Montgomery%2C%20AL","Hilton Garden Inn Montgomery East")</f>
         <v>Hilton Garden Inn Montgomery East</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F14" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>150</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>125</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1534,46 +1528,46 @@
         <v>3</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D15" s="36" t="str">
-        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Courtyard%20Montgomery%20%28Carmichael%29%2C%20Montgomery%2C%20AL","Courtyard Montgomery (Carmichael)")</f>
-        <v>Courtyard Montgomery (Carmichael)</v>
+        <f aca="false">HYPERLINK("https://www.hotels.com/Hotel-Search?destination=Hampton%20Inn%20%26%20Suites%20EastChase%2C%20Montgomery%2C%20AL","Hampton Inn &amp; Suites EastChase")</f>
+        <v>Hampton Inn &amp; Suites EastChase</v>
       </c>
       <c r="E15" s="6" t="s">
         <v>60</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>120</v>
+        <v>168</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="G19" s="28" t="n">
         <f aca="false">SUMIF(A7:A15,"x",G7:G15)</f>
-        <v>398</v>
+        <v>484</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H20" s="13" t="n">
         <f aca="false">SUMIF(A7:A15,"x",G7:G15)*B4</f>
-        <v>796</v>
+        <v>968</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>